<commit_message>
Improve TE calculator: 3-way paint-delivered entry + TE>100% warning
- Fixes the TE>100% trap: paint volume can now be entered via pump/totalizer
  (direct cc), paint weight used (/ rho_mix), or flow x TOTAL paint-on time.
- Adds a SANITY CHECK row and conditional formatting that flags any TE>100%
  in red (impossible - area/DFT too high or paint volume too low).
- Pre-fills Trial 1 with the user's real material and process data
  (paint 1.2 g/cc, VS/WS 57%, 100:50 reduction, area 12.92 m2, DFT 16 um).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hq9x5y2wEsju4khHMmKDpz
</commit_message>
<xml_diff>
--- a/Transfer_Efficiency_Calculator.xlsx
+++ b/Transfer_Efficiency_Calculator.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -103,6 +103,12 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -142,7 +148,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -164,11 +170,55 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -236,26 +286,31 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -264,6 +319,34 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -344,37 +427,62 @@
   <commentList>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
-        <t>Density of the paint as received (before thinning). Typical solvent-borne base/clear ~ 0.95-1.15 g/cc.</t>
+        <t>Density of the paint as received (before thinning).</t>
       </text>
     </comment>
     <comment ref="C8" authorId="0" shapeId="0">
       <text>
-        <t>Volume fraction of the supplied paint that stays as dry film. From the Technical Data Sheet.</t>
+        <t>Volume fraction of supplied paint that stays as dry film (from TDS).</t>
       </text>
     </comment>
     <comment ref="C9" authorId="0" shapeId="0">
       <text>
-        <t>Weight fraction of non-volatiles in the supplied paint. From the Technical Data Sheet.</t>
+        <t>Weight fraction of non-volatiles (from TDS). NOTE: for most paints WS is a bit HIGHER than VS because solids are denser than solvent. You entered WS=VS=57%; only Method A (weight) depends on this - Method B (DFT) does not.</t>
       </text>
     </comment>
     <comment ref="C10" authorId="0" shapeId="0">
       <text>
-        <t>Thinner/solvent density. Assumed 100% volatile (contributes no solids).</t>
+        <t>Thinner density; assumed 100% volatile.</t>
       </text>
     </comment>
     <comment ref="C11" authorId="0" shapeId="0">
       <text>
-        <t>Reduction recipe. e.g. 100:20 -&gt; paint parts = 100.</t>
+        <t>Reduction recipe, e.g. 100:50.</t>
       </text>
     </comment>
     <comment ref="C12" authorId="0" shapeId="0">
       <text>
-        <t>Reduction recipe. e.g. 100:20 -&gt; thinner parts = 20.</t>
+        <t>Reduction recipe, e.g. 100:50.</t>
       </text>
     </comment>
     <comment ref="C17" authorId="0" shapeId="0">
       <text>
-        <t>rho_solids = rho_paint x WS_paint / VS_paint.  This constant bridges the WEIGHT method and the DFT/VOLUME method.</t>
+        <t>rho_solids = rho_paint x WS_paint / VS_paint. Bridges the WEIGHT method and the DFT/VOLUME method.</t>
+      </text>
+    </comment>
+    <comment ref="D32" authorId="0" shapeId="0">
+      <text>
+        <t>THIS is the usual error. For a whole area you must use the TOTAL paint-on time across ALL passes. A single 50 s pass under-counts paint and pushes TE over 100%. Better: use option B (totalizer) or C (paint weight) below.</t>
+      </text>
+    </comment>
+    <comment ref="D33" authorId="0" shapeId="0">
+      <text>
+        <t>Best input: total cc dispensed to the bell over the WHOLE cycle, from the gear-pump / flow totalizer. Leave A blank if you use this.</t>
+      </text>
+    </comment>
+    <comment ref="D34" authorId="0" shapeId="0">
+      <text>
+        <t>Weigh the paint consumed (pot before - after) and the sheet divides by rho_mix to get volume.</t>
+      </text>
+    </comment>
+    <comment ref="D37" authorId="0" shapeId="0">
+      <text>
+        <t>Enter the real cured before-weight for THIS panel. (Left blank - Method A stays empty until you fill W1 and W2.)</t>
+      </text>
+    </comment>
+    <comment ref="D41" authorId="0" shapeId="0">
+      <text>
+        <t>Confirmed correct = 12.92 m2 (whole part).</t>
       </text>
     </comment>
   </commentList>
@@ -670,12 +778,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -686,28 +794,28 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PAINT TRANSFER EFFICIENCY (TE) CALCULATOR  —  Robotic / Bell-Atomizer Solvent-Borne Application</t>
+          <t>PAINT TRANSFER EFFICIENCY (TE) CALCULATOR  -  Robotic / Bell-Atomizer Solvent-Borne Application</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Matches the PRACTICAL foil/gravimetric method (ASTM D5066) with the THEORETICAL DFT/volume-solids method on one sheet. Enter values only in the soft-yellow cells; everything else is auto-calculated.</t>
+          <t>Matches the PRACTICAL foil/gravimetric method (ASTM D5066) with the THEORETICAL DFT/volume-solids method on one sheet. Fill only the soft-yellow cells. TE over 100% is impossible - the sheet flags it in red.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>TE = (paint SOLIDS deposited on part) / (paint SOLIDS sprayed) x 100.   Refs: ASTM D5066 / D5286 / D5327; coverage identity  m2/L = 10 x VS%  /  DFT(um).</t>
+          <t>TE = (paint SOLIDS deposited on part) / (paint SOLIDS sprayed) x 100.   Refs: ASTM D5066 / D5286 / D5327;  coverage identity  m2/L = 10 x VS% / DFT(um).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1)  MATERIAL &amp; MIX PROPERTIES   (global inputs — apply to all trials)</t>
+          <t>1)  MATERIAL &amp; MIX PROPERTIES   (global inputs - apply to all trials)</t>
         </is>
       </c>
     </row>
@@ -745,7 +853,7 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>1.05</v>
+        <v>1.2</v>
       </c>
       <c r="D7" s="10" t="inlineStr"/>
       <c r="E7" s="10" t="inlineStr"/>
@@ -765,7 +873,7 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.22</v>
+        <v>0.57</v>
       </c>
       <c r="D8" s="10" t="inlineStr"/>
       <c r="E8" s="10" t="inlineStr"/>
@@ -785,7 +893,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>0.3</v>
+        <v>0.57</v>
       </c>
       <c r="D9" s="10" t="inlineStr"/>
       <c r="E9" s="10" t="inlineStr"/>
@@ -816,7 +924,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Mix ratio — PAINT parts (by volume)</t>
+          <t>Mix ratio - PAINT parts (by volume)</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -836,7 +944,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Mix ratio — THINNER parts (by volume)</t>
+          <t>Mix ratio - THINNER parts (by volume)</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -845,7 +953,7 @@
         </is>
       </c>
       <c r="C12" s="12" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D12" s="10" t="inlineStr"/>
       <c r="E12" s="10" t="inlineStr"/>
@@ -955,7 +1063,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2)  TRIAL LOG   (one column per spray test — fill yellow input cells; Trial 1 is a worked example)</t>
+          <t>2)  TRIAL LOG   (one column per spray test - Trial 1 pre-filled with your data)</t>
         </is>
       </c>
     </row>
@@ -977,7 +1085,7 @@
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>Trial 1 (example)</t>
+          <t>Trial 1 (yours)</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1004,7 +1112,7 @@
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Process / robot parameters   (logged for correlation — only Flow &amp; Time enter the TE math)</t>
+          <t>Process / robot parameters   (logged for correlation - only paint volume enters the TE math)</t>
         </is>
       </c>
     </row>
@@ -1021,11 +1129,11 @@
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>Atomizer rotation speed</t>
+          <t>atomizer rotation speed</t>
         </is>
       </c>
       <c r="D22" s="12" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E22" s="12" t="n"/>
       <c r="F22" s="12" t="n"/>
@@ -1035,7 +1143,7 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Shaping air — inner (shape-in)</t>
+          <t>Shaping air - inner (shape-in)</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -1045,11 +1153,11 @@
       </c>
       <c r="C23" s="20" t="inlineStr">
         <is>
-          <t>Inner shaping-air flow</t>
+          <t>inner shaping-air flow</t>
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E23" s="12" t="n"/>
       <c r="F23" s="12" t="n"/>
@@ -1059,7 +1167,7 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Shaping air — outer (shape-out)</t>
+          <t>Shaping air - outer (shape-out)</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -1069,7 +1177,7 @@
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>Outer shaping-air flow</t>
+          <t>outer shaping-air flow</t>
         </is>
       </c>
       <c r="D24" s="12" t="n">
@@ -1093,7 +1201,7 @@
       </c>
       <c r="C25" s="20" t="inlineStr">
         <is>
-          <t>Drive/atomizing air</t>
+          <t>drive/atomizing air</t>
         </is>
       </c>
       <c r="D25" s="21" t="n">
@@ -1121,7 +1229,7 @@
         </is>
       </c>
       <c r="D26" s="12" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E26" s="12" t="n"/>
       <c r="F26" s="12" t="n"/>
@@ -1141,11 +1249,11 @@
       </c>
       <c r="C27" s="20" t="inlineStr">
         <is>
-          <t>Stand-off</t>
+          <t>stand-off</t>
         </is>
       </c>
       <c r="D27" s="12" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="E27" s="12" t="n"/>
       <c r="F27" s="12" t="n"/>
@@ -1165,7 +1273,7 @@
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>As-sprayed viscosity</t>
+          <t>as-sprayed viscosity</t>
         </is>
       </c>
       <c r="D28" s="12" t="n">
@@ -1189,11 +1297,11 @@
       </c>
       <c r="C29" s="20" t="inlineStr">
         <is>
-          <t>Paint temp at applicator</t>
+          <t>paint temp at applicator</t>
         </is>
       </c>
       <c r="D29" s="12" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E29" s="12" t="n"/>
       <c r="F29" s="12" t="n"/>
@@ -1201,47 +1309,30 @@
       <c r="H29" s="12" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="inlineStr">
-        <is>
-          <t>Paint FLOW rate  (Q)</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>cc/min</t>
-        </is>
-      </c>
-      <c r="C30" s="20" t="inlineStr">
-        <is>
-          <t>USED IN CALC</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="n">
-        <v>250</v>
-      </c>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="12" t="n"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>PAINT DELIVERED   (enter ONE method; priority  B &gt; C &gt; A)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="22" t="inlineStr">
         <is>
-          <t>Spray TIME  (t)</t>
+          <t>A) Flow rate  (Q)</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>cc/min</t>
         </is>
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
-          <t>USED IN CALC</t>
+          <t>option A: Q x t / 60</t>
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>20</v>
+        <v>350</v>
       </c>
       <c r="E31" s="12" t="n"/>
       <c r="F31" s="12" t="n"/>
@@ -1249,40 +1340,55 @@
       <c r="H31" s="12" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="19" t="inlineStr">
-        <is>
-          <t>Method A — PRACTICAL (gravimetric foil/panel):  weigh BEFORE and AFTER full cure</t>
-        </is>
-      </c>
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>A) Paint-on TIME - TOTAL (all passes)</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>use TOTAL trigger-on time, not one pass</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="12" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Weight BEFORE spraying  (W1)</t>
+          <t>B) Total paint delivered - DIRECT</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cc</t>
         </is>
       </c>
       <c r="C33" s="20" t="inlineStr">
         <is>
-          <t>Foil/panel tare weight</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n"/>
+          <t>option B (pump totalizer) - preferred</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="12" t="n"/>
+      <c r="H33" s="12" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Weight AFTER full cure  (W2)</t>
+          <t>C) Paint USED - by weight</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
@@ -1292,80 +1398,76 @@
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
-          <t>After solvent fully baked off</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="n">
-        <v>31.32</v>
-      </c>
-      <c r="E34" s="9" t="n"/>
-      <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
+          <t>option C: weight / rho_mix</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="21" t="n"/>
+      <c r="F34" s="21" t="n"/>
+      <c r="G34" s="21" t="n"/>
+      <c r="H34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Deposited SOLIDS  Wp = W2 - W1</t>
+          <t>Delivered volume  V</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>cc</t>
         </is>
       </c>
       <c r="C35" s="20" t="inlineStr">
         <is>
-          <t>Wp = W2 - W1</t>
+          <t>picks B, else C/rho_mix, else A</t>
         </is>
       </c>
       <c r="D35" s="23">
-        <f>IF(OR(D33="",D34=""),"",D34-D33)</f>
+        <f>IF(D33&lt;&gt;"",D33,IF(D34&lt;&gt;"",D34/$C$15,IF(D31*D32=0,"",D31*D32/60)))</f>
         <v/>
       </c>
       <c r="E35" s="23">
-        <f>IF(OR(E33="",E34=""),"",E34-E33)</f>
+        <f>IF(E33&lt;&gt;"",E33,IF(E34&lt;&gt;"",E34/$C$15,IF(E31*E32=0,"",E31*E32/60)))</f>
         <v/>
       </c>
       <c r="F35" s="23">
-        <f>IF(OR(F33="",F34=""),"",F34-F33)</f>
+        <f>IF(F33&lt;&gt;"",F33,IF(F34&lt;&gt;"",F34/$C$15,IF(F31*F32=0,"",F31*F32/60)))</f>
         <v/>
       </c>
       <c r="G35" s="23">
-        <f>IF(OR(G33="",G34=""),"",G34-G33)</f>
+        <f>IF(G33&lt;&gt;"",G33,IF(G34&lt;&gt;"",G34/$C$15,IF(G31*G32=0,"",G31*G32/60)))</f>
         <v/>
       </c>
       <c r="H35" s="23">
-        <f>IF(OR(H33="",H34=""),"",H34-H33)</f>
+        <f>IF(H33&lt;&gt;"",H33,IF(H34&lt;&gt;"",H34/$C$15,IF(H31*H32=0,"",H31*H32/60)))</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>Method B — THEORETICAL (DFT x area):  dry-film thickness over the painted area</t>
+          <t>Method A - PRACTICAL (gravimetric foil/panel):  weigh BEFORE and AFTER full cure</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Applied area  (A)</t>
+          <t>Weight BEFORE spraying  (W1)</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>g</t>
         </is>
       </c>
       <c r="C37" s="20" t="inlineStr">
         <is>
-          <t>Area actually coated</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="n">
-        <v>0.6</v>
-      </c>
+          <t>foil/panel tare weight</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="n"/>
       <c r="E37" s="9" t="n"/>
       <c r="F37" s="9" t="n"/>
       <c r="G37" s="9" t="n"/>
@@ -1374,642 +1476,728 @@
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Measured DFT — average  (t_dry)</t>
+          <t>Weight AFTER full cure  (W2)</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>um</t>
+          <t>g</t>
         </is>
       </c>
       <c r="C38" s="20" t="inlineStr">
         <is>
-          <t>Mean of several gauge readings</t>
-        </is>
-      </c>
-      <c r="D38" s="21" t="n">
-        <v>19</v>
-      </c>
-      <c r="E38" s="21" t="n"/>
-      <c r="F38" s="21" t="n"/>
-      <c r="G38" s="21" t="n"/>
-      <c r="H38" s="21" t="n"/>
+          <t>after solvent fully baked off</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="9" t="n"/>
+      <c r="F38" s="9" t="n"/>
+      <c r="G38" s="9" t="n"/>
+      <c r="H38" s="9" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Computed — quantity sprayed</t>
-        </is>
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Deposited SOLIDS  Wp = W2 - W1</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>Wp = W2 - W1</t>
+        </is>
+      </c>
+      <c r="D39" s="24">
+        <f>IF(OR(D37="",D38=""),"",D38-D37)</f>
+        <v/>
+      </c>
+      <c r="E39" s="24">
+        <f>IF(OR(E37="",E38=""),"",E38-E37)</f>
+        <v/>
+      </c>
+      <c r="F39" s="24">
+        <f>IF(OR(F37="",F38=""),"",F38-F37)</f>
+        <v/>
+      </c>
+      <c r="G39" s="24">
+        <f>IF(OR(G37="",G38=""),"",G38-G37)</f>
+        <v/>
+      </c>
+      <c r="H39" s="24">
+        <f>IF(OR(H37="",H38=""),"",H38-H37)</f>
+        <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>Delivered volume  V = Q x t / 60</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>cc</t>
-        </is>
-      </c>
-      <c r="C40" s="20" t="inlineStr">
-        <is>
-          <t>V = Q x t / 60 (as-sprayed mix)</t>
-        </is>
-      </c>
-      <c r="D40" s="24">
-        <f>IF(D30*D31=0,"",D30*D31/60)</f>
-        <v/>
-      </c>
-      <c r="E40" s="24">
-        <f>IF(E30*E31=0,"",E30*E31/60)</f>
-        <v/>
-      </c>
-      <c r="F40" s="24">
-        <f>IF(F30*F31=0,"",F30*F31/60)</f>
-        <v/>
-      </c>
-      <c r="G40" s="24">
-        <f>IF(G30*G31=0,"",G30*G31/60)</f>
-        <v/>
-      </c>
-      <c r="H40" s="24">
-        <f>IF(H30*H31=0,"",H30*H31/60)</f>
-        <v/>
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Method B - THEORETICAL (DFT x area):  dry-film thickness over the painted area</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>SOLIDS sprayed — volume</t>
+          <t>Applied area  (A)</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>cc</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="C41" s="20" t="inlineStr">
         <is>
-          <t>V x VS_mix</t>
-        </is>
-      </c>
-      <c r="D41" s="23">
-        <f>IF(D40="","",D40*$C$14)</f>
-        <v/>
-      </c>
-      <c r="E41" s="23">
-        <f>IF(E40="","",E40*$C$14)</f>
-        <v/>
-      </c>
-      <c r="F41" s="23">
-        <f>IF(F40="","",F40*$C$14)</f>
-        <v/>
-      </c>
-      <c r="G41" s="23">
-        <f>IF(G40="","",G40*$C$14)</f>
-        <v/>
-      </c>
-      <c r="H41" s="23">
-        <f>IF(H40="","",H40*$C$14)</f>
-        <v/>
-      </c>
+          <t>area actually coated</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>12.92</v>
+      </c>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>SOLIDS sprayed — mass</t>
+          <t>Measured DFT - average  (t_dry)</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>um</t>
         </is>
       </c>
       <c r="C42" s="20" t="inlineStr">
         <is>
-          <t>V x rho_mix x WS_mix</t>
-        </is>
-      </c>
-      <c r="D42" s="23">
-        <f>IF(D40="","",D40*$C$15*$C$16)</f>
-        <v/>
-      </c>
-      <c r="E42" s="23">
-        <f>IF(E40="","",E40*$C$15*$C$16)</f>
-        <v/>
-      </c>
-      <c r="F42" s="23">
-        <f>IF(F40="","",F40*$C$15*$C$16)</f>
-        <v/>
-      </c>
-      <c r="G42" s="23">
-        <f>IF(G40="","",G40*$C$15*$C$16)</f>
-        <v/>
-      </c>
-      <c r="H42" s="23">
-        <f>IF(H40="","",H40*$C$15*$C$16)</f>
-        <v/>
-      </c>
+          <t>mean of several gauge readings</t>
+        </is>
+      </c>
+      <c r="D42" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="E42" s="21" t="n"/>
+      <c r="F42" s="21" t="n"/>
+      <c r="G42" s="21" t="n"/>
+      <c r="H42" s="21" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>RESULTS — Transfer Efficiency</t>
+          <t>Computed - quantity sprayed</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="inlineStr">
-        <is>
-          <t>TE — Method A (gravimetric)</t>
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>SOLIDS sprayed - volume</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>cc</t>
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr">
         <is>
-          <t>Wp / solids-mass-sprayed</t>
-        </is>
-      </c>
-      <c r="D44" s="25">
-        <f>IFERROR(D35/D42,"")</f>
-        <v/>
-      </c>
-      <c r="E44" s="25">
-        <f>IFERROR(E35/E42,"")</f>
-        <v/>
-      </c>
-      <c r="F44" s="25">
-        <f>IFERROR(F35/F42,"")</f>
-        <v/>
-      </c>
-      <c r="G44" s="25">
-        <f>IFERROR(G35/G42,"")</f>
-        <v/>
-      </c>
-      <c r="H44" s="25">
-        <f>IFERROR(H35/H42,"")</f>
+          <t>V x VS_mix</t>
+        </is>
+      </c>
+      <c r="D44" s="24">
+        <f>IF(D35="","",D35*$C$14)</f>
+        <v/>
+      </c>
+      <c r="E44" s="24">
+        <f>IF(E35="","",E35*$C$14)</f>
+        <v/>
+      </c>
+      <c r="F44" s="24">
+        <f>IF(F35="","",F35*$C$14)</f>
+        <v/>
+      </c>
+      <c r="G44" s="24">
+        <f>IF(G35="","",G35*$C$14)</f>
+        <v/>
+      </c>
+      <c r="H44" s="24">
+        <f>IF(H35="","",H35*$C$14)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="inlineStr">
-        <is>
-          <t>TE — Method B (DFT / theoretical)</t>
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>SOLIDS sprayed - mass</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>g</t>
         </is>
       </c>
       <c r="C45" s="20" t="inlineStr">
         <is>
-          <t>(A x DFT) / solids-volume-sprayed</t>
-        </is>
-      </c>
-      <c r="D45" s="25">
-        <f>IFERROR((D37*D38)/D41,"")</f>
-        <v/>
-      </c>
-      <c r="E45" s="25">
-        <f>IFERROR((E37*E38)/E41,"")</f>
-        <v/>
-      </c>
-      <c r="F45" s="25">
-        <f>IFERROR((F37*F38)/F41,"")</f>
-        <v/>
-      </c>
-      <c r="G45" s="25">
-        <f>IFERROR((G37*G38)/G41,"")</f>
-        <v/>
-      </c>
-      <c r="H45" s="25">
-        <f>IFERROR((H37*H38)/H41,"")</f>
+          <t>V x rho_mix x WS_mix</t>
+        </is>
+      </c>
+      <c r="D45" s="24">
+        <f>IF(D35="","",D35*$C$15*$C$16)</f>
+        <v/>
+      </c>
+      <c r="E45" s="24">
+        <f>IF(E35="","",E35*$C$15*$C$16)</f>
+        <v/>
+      </c>
+      <c r="F45" s="24">
+        <f>IF(F35="","",F35*$C$15*$C$16)</f>
+        <v/>
+      </c>
+      <c r="G45" s="24">
+        <f>IF(G35="","",G35*$C$15*$C$16)</f>
+        <v/>
+      </c>
+      <c r="H45" s="24">
+        <f>IF(H35="","",H35*$C$15*$C$16)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="22" t="inlineStr">
-        <is>
-          <t>Delta TE  (A - B)</t>
-        </is>
-      </c>
-      <c r="B46" s="8" t="inlineStr">
-        <is>
-          <t>pts</t>
-        </is>
-      </c>
-      <c r="C46" s="20" t="inlineStr">
-        <is>
-          <t>gap between methods (target ~ 0)</t>
-        </is>
-      </c>
-      <c r="D46" s="26">
-        <f>IF(OR(D44="",D45=""),"",D44-D45)</f>
-        <v/>
-      </c>
-      <c r="E46" s="26">
-        <f>IF(OR(E44="",E45=""),"",E44-E45)</f>
-        <v/>
-      </c>
-      <c r="F46" s="26">
-        <f>IF(OR(F44="",F45=""),"",F44-F45)</f>
-        <v/>
-      </c>
-      <c r="G46" s="26">
-        <f>IF(OR(G44="",G45=""),"",G44-G45)</f>
-        <v/>
-      </c>
-      <c r="H46" s="26">
-        <f>IF(OR(H44="",H45=""),"",H44-H45)</f>
-        <v/>
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t>RESULTS - Transfer Efficiency</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="22" t="inlineStr">
         <is>
+          <t>TE - Method A (gravimetric)</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="inlineStr">
+        <is>
+          <t>Wp / solids-mass-sprayed</t>
+        </is>
+      </c>
+      <c r="D47" s="25">
+        <f>IFERROR(D39/D45,"")</f>
+        <v/>
+      </c>
+      <c r="E47" s="25">
+        <f>IFERROR(E39/E45,"")</f>
+        <v/>
+      </c>
+      <c r="F47" s="25">
+        <f>IFERROR(F39/F45,"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="25">
+        <f>IFERROR(G39/G45,"")</f>
+        <v/>
+      </c>
+      <c r="H47" s="25">
+        <f>IFERROR(H39/H45,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>TE - Method B (DFT / theoretical)</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C48" s="20" t="inlineStr">
+        <is>
+          <t>(A x DFT) / solids-volume-sprayed</t>
+        </is>
+      </c>
+      <c r="D48" s="25">
+        <f>IFERROR((D41*D42)/D44,"")</f>
+        <v/>
+      </c>
+      <c r="E48" s="25">
+        <f>IFERROR((E41*E42)/E44,"")</f>
+        <v/>
+      </c>
+      <c r="F48" s="25">
+        <f>IFERROR((F41*F42)/F44,"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="25">
+        <f>IFERROR((G41*G42)/G44,"")</f>
+        <v/>
+      </c>
+      <c r="H48" s="25">
+        <f>IFERROR((H41*H42)/H44,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>Delta TE  (A - B)</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>pts</t>
+        </is>
+      </c>
+      <c r="C49" s="20" t="inlineStr">
+        <is>
+          <t>gap between methods (target ~ 0)</t>
+        </is>
+      </c>
+      <c r="D49" s="26">
+        <f>IF(OR(D47="",D48=""),"",D47-D48)</f>
+        <v/>
+      </c>
+      <c r="E49" s="26">
+        <f>IF(OR(E47="",E48=""),"",E47-E48)</f>
+        <v/>
+      </c>
+      <c r="F49" s="26">
+        <f>IF(OR(F47="",F48=""),"",F47-F48)</f>
+        <v/>
+      </c>
+      <c r="G49" s="26">
+        <f>IF(OR(G47="",G48=""),"",G47-G48)</f>
+        <v/>
+      </c>
+      <c r="H49" s="26">
+        <f>IF(OR(H47="",H48=""),"",H47-H48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="inlineStr">
+        <is>
           <t>Relative difference</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C47" s="20" t="inlineStr">
+      <c r="C50" s="20" t="inlineStr">
         <is>
           <t>(A - B) / B</t>
         </is>
       </c>
-      <c r="D47" s="26">
-        <f>IFERROR((D44-D45)/D45,"")</f>
-        <v/>
-      </c>
-      <c r="E47" s="26">
-        <f>IFERROR((E44-E45)/E45,"")</f>
-        <v/>
-      </c>
-      <c r="F47" s="26">
-        <f>IFERROR((F44-F45)/F45,"")</f>
-        <v/>
-      </c>
-      <c r="G47" s="26">
-        <f>IFERROR((G44-G45)/G45,"")</f>
-        <v/>
-      </c>
-      <c r="H47" s="26">
-        <f>IFERROR((H44-H45)/H45,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="19" t="inlineStr">
-        <is>
-          <t>RECONCILIATION — match theory vs practice</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>Deposited solids volume (from DFT)</t>
-        </is>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>cc</t>
-        </is>
-      </c>
-      <c r="C49" s="20" t="inlineStr">
-        <is>
-          <t>A x DFT</t>
-        </is>
-      </c>
-      <c r="D49" s="23">
-        <f>IF(OR(D37="",D38=""),"",D37*D38)</f>
-        <v/>
-      </c>
-      <c r="E49" s="23">
-        <f>IF(OR(E37="",E38=""),"",E37*E38)</f>
-        <v/>
-      </c>
-      <c r="F49" s="23">
-        <f>IF(OR(F37="",F38=""),"",F37*F38)</f>
-        <v/>
-      </c>
-      <c r="G49" s="23">
-        <f>IF(OR(G37="",G38=""),"",G37*G38)</f>
-        <v/>
-      </c>
-      <c r="H49" s="23">
-        <f>IF(OR(H37="",H38=""),"",H37*H38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>DFT predicted from WEIGHT</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="inlineStr">
-        <is>
-          <t>um</t>
-        </is>
-      </c>
-      <c r="C50" s="20" t="inlineStr">
-        <is>
-          <t>Wp / (rho_solids x A)</t>
-        </is>
-      </c>
-      <c r="D50" s="27">
-        <f>IFERROR(D35/($C$17*D37),"")</f>
-        <v/>
-      </c>
-      <c r="E50" s="27">
-        <f>IFERROR(E35/($C$17*E37),"")</f>
-        <v/>
-      </c>
-      <c r="F50" s="27">
-        <f>IFERROR(F35/($C$17*F37),"")</f>
-        <v/>
-      </c>
-      <c r="G50" s="27">
-        <f>IFERROR(G35/($C$17*G37),"")</f>
-        <v/>
-      </c>
-      <c r="H50" s="27">
-        <f>IFERROR(H35/($C$17*H37),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>DFT match  (predicted - measured)</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>um</t>
-        </is>
-      </c>
+      <c r="D50" s="26">
+        <f>IFERROR((D47-D48)/D48,"")</f>
+        <v/>
+      </c>
+      <c r="E50" s="26">
+        <f>IFERROR((E47-E48)/E48,"")</f>
+        <v/>
+      </c>
+      <c r="F50" s="26">
+        <f>IFERROR((F47-F48)/F48,"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="26">
+        <f>IFERROR((G47-G48)/G48,"")</f>
+        <v/>
+      </c>
+      <c r="H50" s="26">
+        <f>IFERROR((H47-H48)/H48,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>SANITY CHECK</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr"/>
       <c r="C51" s="20" t="inlineStr">
         <is>
-          <t>cross-check of the two methods (~ 0)</t>
-        </is>
-      </c>
-      <c r="D51" s="27">
-        <f>IF(OR(D50="",D38=""),"",D50-D38)</f>
-        <v/>
-      </c>
-      <c r="E51" s="27">
-        <f>IF(OR(E50="",E38=""),"",E50-E38)</f>
-        <v/>
-      </c>
-      <c r="F51" s="27">
-        <f>IF(OR(F50="",F38=""),"",F50-F38)</f>
-        <v/>
-      </c>
-      <c r="G51" s="27">
-        <f>IF(OR(G50="",G38=""),"",G50-G38)</f>
-        <v/>
-      </c>
-      <c r="H51" s="27">
-        <f>IF(OR(H50="",H38=""),"",H50-H38)</f>
-        <v/>
-      </c>
+          <t>auto-flags impossible results</t>
+        </is>
+      </c>
+      <c r="D51" s="28">
+        <f>IF(D48="","",IF(D48&gt;1,"CHECK: TE(B)&gt;100% - area/DFT too high OR paint volume too low",IF(AND(ISNUMBER(D47),D47&gt;1),"CHECK: TE(A)&gt;100%",IF(AND(ISNUMBER(D47),ABS(D47-D48)&gt;0.1),"Methods disagree &gt;10 pts - check data","OK"))))</f>
+        <v/>
+      </c>
+      <c r="E51" s="29" t="n"/>
+      <c r="F51" s="29" t="n"/>
+      <c r="G51" s="29" t="n"/>
+      <c r="H51" s="30" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>Theoretical coverage @ measured DFT</t>
-        </is>
-      </c>
-      <c r="B52" s="8" t="inlineStr">
-        <is>
-          <t>m2/L</t>
-        </is>
-      </c>
-      <c r="C52" s="20" t="inlineStr">
-        <is>
-          <t>10 x VS% / DFT  (at 100% TE)</t>
-        </is>
-      </c>
-      <c r="D52" s="24">
-        <f>IFERROR(1000*$C$14/D38,"")</f>
-        <v/>
-      </c>
-      <c r="E52" s="24">
-        <f>IFERROR(1000*$C$14/E38,"")</f>
-        <v/>
-      </c>
-      <c r="F52" s="24">
-        <f>IFERROR(1000*$C$14/F38,"")</f>
-        <v/>
-      </c>
-      <c r="G52" s="24">
-        <f>IFERROR(1000*$C$14/G38,"")</f>
-        <v/>
-      </c>
-      <c r="H52" s="24">
-        <f>IFERROR(1000*$C$14/H38,"")</f>
-        <v/>
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>RECONCILIATION - match theory vs practice</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Practical coverage achieved</t>
+          <t>Deposited solids volume (from DFT)</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>m2/L</t>
+          <t>cc</t>
         </is>
       </c>
       <c r="C53" s="20" t="inlineStr">
         <is>
-          <t>A x 1000 / V</t>
+          <t>A x DFT</t>
         </is>
       </c>
       <c r="D53" s="24">
-        <f>IFERROR(D37*1000/D40,"")</f>
+        <f>IF(OR(D41="",D42=""),"",D41*D42)</f>
         <v/>
       </c>
       <c r="E53" s="24">
-        <f>IFERROR(E37*1000/E40,"")</f>
+        <f>IF(OR(E41="",E42=""),"",E41*E42)</f>
         <v/>
       </c>
       <c r="F53" s="24">
-        <f>IFERROR(F37*1000/F40,"")</f>
+        <f>IF(OR(F41="",F42=""),"",F41*F42)</f>
         <v/>
       </c>
       <c r="G53" s="24">
-        <f>IFERROR(G37*1000/G40,"")</f>
+        <f>IF(OR(G41="",G42=""),"",G41*G42)</f>
         <v/>
       </c>
       <c r="H53" s="24">
-        <f>IFERROR(H37*1000/H40,"")</f>
+        <f>IF(OR(H41="",H42=""),"",H41*H42)</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
+          <t>DFT predicted from WEIGHT</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>um</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>Wp / (rho_solids x A)</t>
+        </is>
+      </c>
+      <c r="D54" s="31">
+        <f>IFERROR(D39/($C$17*D41),"")</f>
+        <v/>
+      </c>
+      <c r="E54" s="31">
+        <f>IFERROR(E39/($C$17*E41),"")</f>
+        <v/>
+      </c>
+      <c r="F54" s="31">
+        <f>IFERROR(F39/($C$17*F41),"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="31">
+        <f>IFERROR(G39/($C$17*G41),"")</f>
+        <v/>
+      </c>
+      <c r="H54" s="31">
+        <f>IFERROR(H39/($C$17*H41),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>DFT match  (predicted - measured)</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>um</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>cross-check of the two methods (~ 0)</t>
+        </is>
+      </c>
+      <c r="D55" s="31">
+        <f>IF(OR(D54="",D42=""),"",D54-D42)</f>
+        <v/>
+      </c>
+      <c r="E55" s="31">
+        <f>IF(OR(E54="",E42=""),"",E54-E42)</f>
+        <v/>
+      </c>
+      <c r="F55" s="31">
+        <f>IF(OR(F54="",F42=""),"",F54-F42)</f>
+        <v/>
+      </c>
+      <c r="G55" s="31">
+        <f>IF(OR(G54="",G42=""),"",G54-G42)</f>
+        <v/>
+      </c>
+      <c r="H55" s="31">
+        <f>IF(OR(H54="",H42=""),"",H54-H42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Theoretical coverage @ measured DFT</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>m2/L</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>10 x VS% / DFT  (at 100% TE)</t>
+        </is>
+      </c>
+      <c r="D56" s="23">
+        <f>IFERROR(1000*$C$14/D42,"")</f>
+        <v/>
+      </c>
+      <c r="E56" s="23">
+        <f>IFERROR(1000*$C$14/E42,"")</f>
+        <v/>
+      </c>
+      <c r="F56" s="23">
+        <f>IFERROR(1000*$C$14/F42,"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="23">
+        <f>IFERROR(1000*$C$14/G42,"")</f>
+        <v/>
+      </c>
+      <c r="H56" s="23">
+        <f>IFERROR(1000*$C$14/H42,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Practical coverage achieved</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>m2/L</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>A x 1000 / V</t>
+        </is>
+      </c>
+      <c r="D57" s="23">
+        <f>IFERROR(D41*1000/D35,"")</f>
+        <v/>
+      </c>
+      <c r="E57" s="23">
+        <f>IFERROR(E41*1000/E35,"")</f>
+        <v/>
+      </c>
+      <c r="F57" s="23">
+        <f>IFERROR(F41*1000/F35,"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="23">
+        <f>IFERROR(G41*1000/G35,"")</f>
+        <v/>
+      </c>
+      <c r="H57" s="23">
+        <f>IFERROR(H41*1000/H35,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
           <t>Coverage-ratio TE  (self-check = Method B)</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C54" s="20" t="inlineStr">
+      <c r="C58" s="20" t="inlineStr">
         <is>
           <t>practical / theoretical</t>
         </is>
       </c>
-      <c r="D54" s="28">
-        <f>IFERROR(D53/D52,"")</f>
-        <v/>
-      </c>
-      <c r="E54" s="28">
-        <f>IFERROR(E53/E52,"")</f>
-        <v/>
-      </c>
-      <c r="F54" s="28">
-        <f>IFERROR(F53/F52,"")</f>
-        <v/>
-      </c>
-      <c r="G54" s="28">
-        <f>IFERROR(G53/G52,"")</f>
-        <v/>
-      </c>
-      <c r="H54" s="28">
-        <f>IFERROR(H53/H52,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="D58" s="32">
+        <f>IFERROR(D57/D56,"")</f>
+        <v/>
+      </c>
+      <c r="E58" s="32">
+        <f>IFERROR(E57/E56,"")</f>
+        <v/>
+      </c>
+      <c r="F58" s="32">
+        <f>IFERROR(F57/F56,"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="32">
+        <f>IFERROR(G57/G56,"")</f>
+        <v/>
+      </c>
+      <c r="H58" s="32">
+        <f>IFERROR(H57/H56,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>HOW TO USE  &amp;  HOW THE TWO METHODS MATCH</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="26" customHeight="1">
-      <c r="A57" s="29" t="inlineStr">
+    <row r="61" ht="26" customHeight="1">
+      <c r="A61" s="28" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
-      <c r="B57" s="30" t="inlineStr">
-        <is>
-          <t>Soft-YELLOW cell = you type here (blue text).  Plain cell = auto-calculated.  Green = the TE result.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="39" customHeight="1">
-      <c r="A58" s="29" t="inlineStr">
-        <is>
-          <t>Method A (practical / foil):</t>
-        </is>
-      </c>
-      <c r="B58" s="30" t="inlineStr">
-        <is>
-          <t>Cover the part/panel with aluminium foil (ASTM D5066).  Weigh = W1.  Spray with the robot, logging every process parameter above.  Bake/cure until ALL solvent is gone.  Re-weigh = W2.  Deposited dry solids = W2 - W1.  TE(A) = (W2 - W1) / solids-mass-sprayed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="39" customHeight="1">
-      <c r="A59" s="29" t="inlineStr">
-        <is>
-          <t>Method B (theoretical / DFT):</t>
-        </is>
-      </c>
-      <c r="B59" s="30" t="inlineStr">
-        <is>
-          <t>Measure the coated area A and the average dry-film thickness (several gauge points).  Because 1 m2 x 1 um = 1 cc, the deposited solids volume = A x DFT.  TE(B) = (A x DFT) / solids-volume-sprayed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="52" customHeight="1">
-      <c r="A60" s="29" t="inlineStr">
+      <c r="B61" s="33" t="inlineStr">
+        <is>
+          <t>Soft-YELLOW = you type here (blue text). Plain = auto-calculated. Green = the TE result. Red = an impossible value to fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="52" customHeight="1">
+      <c r="A62" s="28" t="inlineStr">
+        <is>
+          <t>Paint delivered (KEY):</t>
+        </is>
+      </c>
+      <c r="B62" s="33" t="inlineStr">
+        <is>
+          <t>V must be ALL the mixed paint sprayed while coating area A. Best: option B = pump/totalizer cc over the whole cycle. Or option C = paint weight used / rho_mix. Only use A = flow x time if 'time' is the TOTAL trigger-on time for every pass. A single-pass time is the #1 cause of TE &gt; 100%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="26" customHeight="1">
+      <c r="A63" s="28" t="inlineStr">
+        <is>
+          <t>Method A (practical/foil):</t>
+        </is>
+      </c>
+      <c r="B63" s="33" t="inlineStr">
+        <is>
+          <t>Foil the panel (ASTM D5066), weigh = W1, spray, bake until ALL solvent is gone, re-weigh = W2. Deposited dry solids = W2 - W1.  TE(A) = (W2 - W1) / solids-mass-sprayed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="26" customHeight="1">
+      <c r="A64" s="28" t="inlineStr">
+        <is>
+          <t>Method B (theoretical/DFT):</t>
+        </is>
+      </c>
+      <c r="B64" s="33" t="inlineStr">
+        <is>
+          <t>Measure coated area A and average DFT. Because 1 m2 x 1 um = 1 cc, deposited solids volume = A x DFT.  TE(B) = (A x DFT) / solids-volume-sprayed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="39" customHeight="1">
+      <c r="A65" s="28" t="inlineStr">
         <is>
           <t>Why they match:</t>
         </is>
       </c>
-      <c r="B60" s="30" t="inlineStr">
-        <is>
-          <t>Both estimate the SAME thing - the fraction of sprayed solids that landed on the part - just via mass vs volume.  They are linked by rho_solids (row 17).  If TE(A) = TE(B) and 'DFT predicted from weight' = 'measured DFT', your data is internally consistent.  A large Delta TE flags a bad weight, wrong solids %, mis-measured area, or solvent not fully baked off.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="29" t="inlineStr">
-        <is>
-          <t>Solids sprayed:</t>
-        </is>
-      </c>
-      <c r="B61" s="30" t="inlineStr">
-        <is>
-          <t>Delivered volume V = Q x t / 60.  It is the AS-SPRAYED (thinned) material, so the sheet uses the mixed VS_mix / WS_mix / rho_mix from Section 1 - not the neat-paint values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="29" t="inlineStr">
+      <c r="B65" s="33" t="inlineStr">
+        <is>
+          <t>Both estimate the same fraction of sprayed solids that landed on the part - one via mass, one via volume - linked by rho_solids (row 17). If TE(A) = TE(B) and 'DFT predicted from weight' = 'measured DFT', the data is consistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="26" customHeight="1">
+      <c r="A66" s="28" t="inlineStr">
+        <is>
+          <t>Quick check:</t>
+        </is>
+      </c>
+      <c r="B66" s="33" t="inlineStr">
+        <is>
+          <t>For a fixed A, DFT and VS_mix:  TE = (A x DFT / VS_mix) / V.  Larger true V -&gt; lower (real) TE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="A67" s="28" t="inlineStr">
         <is>
           <t>Typical TE:</t>
         </is>
       </c>
-      <c r="B62" s="30" t="inlineStr">
-        <is>
-          <t>Air-spray ~25-40%, HVLP ~45-65%, electrostatic bell ~70-95% (higher voltage / lower flow / correct shaping air raise TE).</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="15" customHeight="1">
-      <c r="A63" s="29" t="inlineStr">
-        <is>
-          <t>Caveat:</t>
-        </is>
-      </c>
-      <c r="B63" s="30" t="inlineStr">
-        <is>
-          <t>Weigh W2 only after the film is FULLY cured; a wet weight includes solvent and overstates TE.</t>
+      <c r="B67" s="33" t="inlineStr">
+        <is>
+          <t>Air-spray ~25-40%, HVLP ~45-65%, electrostatic bell ~70-95%.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A39:H39"/>
+  <mergeCells count="21">
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="B65:H65"/>
+    <mergeCell ref="A60:H60"/>
     <mergeCell ref="A36:H36"/>
+    <mergeCell ref="B64:H64"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B63:H63"/>
     <mergeCell ref="B62:H62"/>
-    <mergeCell ref="B59:H59"/>
-    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="B66:H66"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A21:H21"/>
-    <mergeCell ref="B58:H58"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="B60:H60"/>
+    <mergeCell ref="B67:H67"/>
     <mergeCell ref="B61:H61"/>
-    <mergeCell ref="B57:H57"/>
     <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="D51:H51"/>
     <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
+  <conditionalFormatting sqref="D47:H48">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D51:H51">
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>LEFT(D51,5)="CHECK"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>